<commit_message>
Align C3DC regression with QA Explore filters and expected data
</commit_message>
<xml_diff>
--- a/InputFiles/C3DC/TC01_C3DC_phs000469_SexAtBirth-Male.xlsx
+++ b/InputFiles/C3DC/TC01_C3DC_phs000469_SexAtBirth-Male.xlsx
@@ -536,7 +536,7 @@
 OPTIONAL MATCH (sm:sample)-[:of_sample]-&gt;(:participant)-[:of_participant]-&gt;(:consent_group)-[:of_consent_group]-&gt;(s)
 WITH s, num_of_participants, count(DISTINCT sm) AS num_of_samples
 OPTIONAL MATCH (d:diagnosis)-[:of_diagnosis]-&gt;(dp:participant)-[:of_participant]-&gt;(:consent_group)-[:of_consent_group]-&gt;(s)
-WITH s, num_of_participants, num_of_samples, d.diagnosis AS diagnosis_name, count(DISTINCT dp) AS diagnosis_n
+WITH s, num_of_participants, num_of_samples, d.diagnosis AS diagnosis_name, count(d) AS diagnosis_n
 ORDER BY diagnosis_n DESC, diagnosis_name DESC
 WITH s, num_of_participants, num_of_samples,
      [item IN collect(CASE WHEN diagnosis_name IS NULL THEN null ELSE diagnosis_name + ' (' + toString(diagnosis_n) + ')' END) WHERE item IS NOT NULL] AS diagnosis_all
@@ -549,13 +549,13 @@
   WHEN size(coalesce(d2.anatomic_site, [])) = 0 THEN [null]
   ELSE d2.anatomic_site
 END AS site_raw
-WITH s, num_of_participants, num_of_samples, diagnosis_items, diagnosis_more, d2, site_raw,
+WITH s, num_of_participants, num_of_samples, diagnosis_items, diagnosis_more, site_raw,
      CASE
        WHEN site_raw IS NULL OR trim(toString(site_raw)) = '' THEN 'Not Reported'
        ELSE site_raw
      END AS site
-WITH s, num_of_participants, num_of_samples, diagnosis_items, diagnosis_more, site, count(DISTINCT d2) AS site_n
-ORDER BY site_n DESC, site ASC
+WITH s, num_of_participants, num_of_samples, diagnosis_items, diagnosis_more, site, count(*) AS site_n
+ORDER BY site_n DESC, site DESC
 WITH s, num_of_participants, num_of_samples, diagnosis_items, diagnosis_more,
      collect(site + ' (' + toString(site_n) + ')') AS site_all
 WITH s, num_of_participants, num_of_samples, diagnosis_items, diagnosis_more,
@@ -610,6 +610,9 @@
           <t>MATCH (d:diagnosis)-[:of_diagnosis]-&gt;(p:participant)-[:of_participant]-&gt;(:consent_group)-[:of_consent_group]-&gt;(s:study)
 WHERE s.dbgap_accession = 'phs000469'
   AND p.sex_at_birth = 'Male'
+WITH p, s, d
+ORDER BY p.participant_id, d.diagnosis_id DESC
+WITH p, s, collect(d)[0] AS d
 RETURN p.participant_id AS `Participant ID`,
        d.diagnosis_id AS `Diagnosis ID`,
        d.diagnosis AS `Diagnosis`,
@@ -674,8 +677,8 @@
          t.treatment_chemotherapy_id AS treatment_id,
          CASE WHEN t.age_at_treatment_start IS NULL OR t.age_at_treatment_start = -999 THEN 'Not Reported' ELSE toString(t.age_at_treatment_start) END AS age_start,
          CASE WHEN t.age_at_treatment_end IS NULL OR t.age_at_treatment_end = -999 THEN 'Not Reported' ELSE toString(t.age_at_treatment_end) END AS age_end,
-         reduce(text = '', item IN coalesce(t.treatment_type, []) | CASE WHEN text = '' THEN item ELSE text + ', ' + item END) AS treatment_type,
-         reduce(text = '', item IN coalesce(t.chemotherapy_agent, []) | CASE WHEN text = '' THEN item ELSE text + ', ' + item END) AS treatment_agent,
+         reduce(text = '', item IN coalesce(t.treatment_type, []) | CASE WHEN text = '' THEN item ELSE text + '; ' + item END) AS treatment_type,
+         reduce(text = '', item IN coalesce(t.chemotherapy_agent, []) | CASE WHEN text = '' THEN item ELSE text + '; ' + item END) AS treatment_agent,
          s.dbgap_accession AS dbgap_accession
   UNION
   MATCH (t:treatment_radiation)-[:of_treatment_radiation]-&gt;(p:participant)-[:of_participant]-&gt;(:consent_group)-[:of_consent_group]-&gt;(s:study)
@@ -684,8 +687,8 @@
          t.treatment_radiation_id AS treatment_id,
          CASE WHEN t.age_at_treatment_start IS NULL OR t.age_at_treatment_start = -999 THEN 'Not Reported' ELSE toString(t.age_at_treatment_start) END AS age_start,
          CASE WHEN t.age_at_treatment_end IS NULL OR t.age_at_treatment_end = -999 THEN 'Not Reported' ELSE toString(t.age_at_treatment_end) END AS age_end,
-         reduce(text = '', item IN coalesce(t.treatment_type, []) | CASE WHEN text = '' THEN item ELSE text + ', ' + item END) AS treatment_type,
-         reduce(text = '', item IN coalesce(t.radiation_therapy_type, []) | CASE WHEN text = '' THEN item ELSE text + ', ' + item END) AS treatment_agent,
+         reduce(text = '', item IN coalesce(t.treatment_type, []) | CASE WHEN text = '' THEN item ELSE text + '; ' + item END) AS treatment_type,
+         reduce(text = '', item IN coalesce(t.radiation_therapy_type, []) | CASE WHEN text = '' THEN item ELSE text + '; ' + item END) AS treatment_agent,
          s.dbgap_accession AS dbgap_accession
   UNION
   MATCH (t:treatment_surgery)-[:of_treatment_surgery]-&gt;(p:participant)-[:of_participant]-&gt;(:consent_group)-[:of_consent_group]-&gt;(s:study)
@@ -694,8 +697,8 @@
          t.treatment_surgery_id AS treatment_id,
          CASE WHEN t.age_at_treatment_start IS NULL OR t.age_at_treatment_start = -999 THEN 'Not Reported' ELSE toString(t.age_at_treatment_start) END AS age_start,
          CASE WHEN t.age_at_treatment_end IS NULL OR t.age_at_treatment_end = -999 THEN 'Not Reported' ELSE toString(t.age_at_treatment_end) END AS age_end,
-         reduce(text = '', item IN coalesce(t.treatment_type, []) | CASE WHEN text = '' THEN item ELSE text + ', ' + item END) AS treatment_type,
-         reduce(text = '', item IN coalesce(t.surgery_type, []) | CASE WHEN text = '' THEN item ELSE text + ', ' + item END) AS treatment_agent,
+         reduce(text = '', item IN coalesce(t.treatment_type, []) | CASE WHEN text = '' THEN item ELSE text + '; ' + item END) AS treatment_type,
+         reduce(text = '', item IN coalesce(t.surgery_type, []) | CASE WHEN text = '' THEN item ELSE text + '; ' + item END) AS treatment_agent,
          s.dbgap_accession AS dbgap_accession
   UNION
   MATCH (t:treatment_other)-[:of_treatment_other]-&gt;(p:participant)-[:of_participant]-&gt;(:consent_group)-[:of_consent_group]-&gt;(s:study)
@@ -704,8 +707,8 @@
          t.treatment_other_id AS treatment_id,
          CASE WHEN t.age_at_treatment_start IS NULL OR t.age_at_treatment_start = -999 THEN 'Not Reported' ELSE toString(t.age_at_treatment_start) END AS age_start,
          CASE WHEN t.age_at_treatment_end IS NULL OR t.age_at_treatment_end = -999 THEN 'Not Reported' ELSE toString(t.age_at_treatment_end) END AS age_end,
-         reduce(text = '', item IN coalesce(t.treatment_type, []) | CASE WHEN text = '' THEN item ELSE text + ', ' + item END) AS treatment_type,
-         reduce(text = '', item IN coalesce(t.other_treatment_type, []) | CASE WHEN text = '' THEN item ELSE text + ', ' + item END) AS treatment_agent,
+         reduce(text = '', item IN coalesce(t.treatment_type, []) | CASE WHEN text = '' THEN item ELSE text + '; ' + item END) AS treatment_type,
+         reduce(text = '', item IN coalesce(t.other_treatment_type, []) | CASE WHEN text = '' THEN item ELSE text + '; ' + item END) AS treatment_agent,
          s.dbgap_accession AS dbgap_accession
 }
 RETURN participant_id AS `Participant ID`,
@@ -713,7 +716,7 @@
        age_start AS `Age at Treatment Start`,
        age_end AS `Age at Treatment End`,
        treatment_type AS `Treatment Type`,
-       treatment_agent AS `Treatment Agent`,
+       CASE WHEN treatment_agent IS NULL OR trim(treatment_agent) = '' THEN 'Not Reported' ELSE treatment_agent END AS `Treatment Agent`,
        dbgap_accession AS `dbGaP Accession`
 ORDER BY treatment_id
 LIMIT 100;</t>

</xml_diff>